<commit_message>
Reestructura OTO MELARA en módulos app logic y word_generator
</commit_message>
<xml_diff>
--- a/data/excelplantilla.xlsx
+++ b/data/excelplantilla.xlsx
@@ -5,15 +5,16 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jesus\curso pandas\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jesus\curso pandas\IG_project\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D6076ACB-AB6F-4FE5-B260-C7403205DA62}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5BC29DF7-EC5D-4852-BD39-2DBCB729B57F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2130" yWindow="2790" windowWidth="21600" windowHeight="11295" xr2:uid="{BCDE5258-4E93-4804-8128-842F739F217B}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{BCDE5258-4E93-4804-8128-842F739F217B}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="OTO MELARA" sheetId="1" r:id="rId1"/>
+    <sheet name="G.M. Rompedora y fumígena" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -25,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="11">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="19">
   <si>
     <t>V1</t>
   </si>
@@ -42,12 +43,6 @@
     <t>PMEDIA</t>
   </si>
   <si>
-    <t>PI</t>
-  </si>
-  <si>
-    <t>PII</t>
-  </si>
-  <si>
     <t>Espoleta</t>
   </si>
   <si>
@@ -58,6 +53,36 @@
   </si>
   <si>
     <t>Fallo</t>
+  </si>
+  <si>
+    <t>P1</t>
+  </si>
+  <si>
+    <t>P2</t>
+  </si>
+  <si>
+    <t>CARGA 1</t>
+  </si>
+  <si>
+    <t>CARGA MÁXIMA</t>
+  </si>
+  <si>
+    <t>VMED (C1)</t>
+  </si>
+  <si>
+    <t>V1 (C1)</t>
+  </si>
+  <si>
+    <t>V2 (C1)</t>
+  </si>
+  <si>
+    <t>V1 (CMAX)</t>
+  </si>
+  <si>
+    <t>V2 (CMAX)</t>
+  </si>
+  <si>
+    <t>VMED (CMAX)</t>
   </si>
 </sst>
 </file>
@@ -461,19 +486,19 @@
         <v>3</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="I1" s="1" t="s">
         <v>4</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="K1" s="1" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
     </row>
     <row r="2" spans="3:11" x14ac:dyDescent="0.25">
@@ -499,10 +524,10 @@
         <v>3029.8150000000001</v>
       </c>
       <c r="J2" s="4" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="K2" s="4" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
     </row>
     <row r="3" spans="3:11" x14ac:dyDescent="0.25">
@@ -528,10 +553,10 @@
         <v>3119.76</v>
       </c>
       <c r="J3" s="4" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="K3" s="4" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
     </row>
     <row r="4" spans="3:11" x14ac:dyDescent="0.25">
@@ -557,10 +582,10 @@
         <v>3060.0749999999998</v>
       </c>
       <c r="J4" s="4" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="K4" s="4" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
     </row>
     <row r="5" spans="3:11" x14ac:dyDescent="0.25">
@@ -586,10 +611,10 @@
         <v>3057.1000000000004</v>
       </c>
       <c r="J5" s="4" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="K5" s="4" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
     </row>
     <row r="6" spans="3:11" x14ac:dyDescent="0.25">
@@ -615,10 +640,53 @@
         <v>2998.4949999999999</v>
       </c>
       <c r="J6" s="4" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="K6" s="4" t="s">
-        <v>9</v>
+        <v>7</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{298C37D3-CA03-4C85-9F91-82C86E07EA81}">
+  <dimension ref="A1:Z1"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="5" max="5" width="10.7109375" customWidth="1"/>
+    <col min="22" max="22" width="15.85546875" customWidth="1"/>
+    <col min="24" max="24" width="13.28515625" customWidth="1"/>
+    <col min="25" max="25" width="11.7109375" customWidth="1"/>
+    <col min="26" max="26" width="15.140625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:26" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>11</v>
+      </c>
+      <c r="C1" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1" t="s">
+        <v>15</v>
+      </c>
+      <c r="E1" t="s">
+        <v>13</v>
+      </c>
+      <c r="V1" t="s">
+        <v>12</v>
+      </c>
+      <c r="X1" t="s">
+        <v>16</v>
+      </c>
+      <c r="Y1" t="s">
+        <v>17</v>
+      </c>
+      <c r="Z1" t="s">
+        <v>18</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
IG10: Nuevo módulo municion_105_51 (VRC/Centauro)
</commit_message>
<xml_diff>
--- a/data/excelplantilla.xlsx
+++ b/data/excelplantilla.xlsx
@@ -8,13 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jesus\curso pandas\IG_project\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5BC29DF7-EC5D-4852-BD39-2DBCB729B57F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{15698755-4C0F-4772-A825-2121597D18F1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{BCDE5258-4E93-4804-8128-842F739F217B}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{BCDE5258-4E93-4804-8128-842F739F217B}"/>
   </bookViews>
   <sheets>
     <sheet name="OTO MELARA" sheetId="1" r:id="rId1"/>
-    <sheet name="G.M. Rompedora y fumígena" sheetId="2" r:id="rId2"/>
+    <sheet name="105_51" sheetId="3" r:id="rId2"/>
+    <sheet name="G.M. Rompedora y fumígena" sheetId="2" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -26,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="19">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="83" uniqueCount="24">
   <si>
     <t>V1</t>
   </si>
@@ -52,9 +53,6 @@
     <t>Correcto</t>
   </si>
   <si>
-    <t>Fallo</t>
-  </si>
-  <si>
     <t>P1</t>
   </si>
   <si>
@@ -83,6 +81,24 @@
   </si>
   <si>
     <t>VMED (CMAX)</t>
+  </si>
+  <si>
+    <t>Serie</t>
+  </si>
+  <si>
+    <t>Vuelo</t>
+  </si>
+  <si>
+    <t>tiempo_traza</t>
+  </si>
+  <si>
+    <t>Vo=1173m/s</t>
+  </si>
+  <si>
+    <t>separacion_partes_metalicas</t>
+  </si>
+  <si>
+    <t>fallo</t>
   </si>
 </sst>
 </file>
@@ -98,7 +114,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -108,6 +124,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF00B050"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -139,7 +161,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1" applyProtection="1">
@@ -150,6 +172,8 @@
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -464,15 +488,17 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BC735DEB-C7CC-4B78-AECF-CBD040F45BCD}">
-  <dimension ref="C1:K6"/>
+  <dimension ref="C1:M6"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="3" max="3" width="12.28515625" customWidth="1"/>
     <col min="6" max="6" width="21.42578125" customWidth="1"/>
     <col min="8" max="8" width="17.140625" customWidth="1"/>
+    <col min="12" max="12" width="28.28515625" customWidth="1"/>
+    <col min="13" max="13" width="16.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="3:11" x14ac:dyDescent="0.25">
+    <row r="1" spans="3:13" x14ac:dyDescent="0.25">
       <c r="C1" s="1" t="s">
         <v>0</v>
       </c>
@@ -486,10 +512,10 @@
         <v>3</v>
       </c>
       <c r="G1" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="H1" s="1" t="s">
         <v>9</v>
-      </c>
-      <c r="H1" s="1" t="s">
-        <v>10</v>
       </c>
       <c r="I1" s="1" t="s">
         <v>4</v>
@@ -500,8 +526,14 @@
       <c r="K1" s="1" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="2" spans="3:11" x14ac:dyDescent="0.25">
+      <c r="L1" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="M1" s="6" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="2" spans="3:13" x14ac:dyDescent="0.25">
       <c r="C2" s="2">
         <v>916.42</v>
       </c>
@@ -530,7 +562,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="3" spans="3:11" x14ac:dyDescent="0.25">
+    <row r="3" spans="3:13" x14ac:dyDescent="0.25">
       <c r="C3" s="2">
         <v>916.49</v>
       </c>
@@ -559,7 +591,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="4" spans="3:11" x14ac:dyDescent="0.25">
+    <row r="4" spans="3:13" x14ac:dyDescent="0.25">
       <c r="C4" s="2">
         <v>915.24</v>
       </c>
@@ -588,7 +620,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="5" spans="3:11" x14ac:dyDescent="0.25">
+    <row r="5" spans="3:13" x14ac:dyDescent="0.25">
       <c r="C5" s="2">
         <v>914.07</v>
       </c>
@@ -611,13 +643,13 @@
         <v>3057.1000000000004</v>
       </c>
       <c r="J5" s="4" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="K5" s="4" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="6" spans="3:11" x14ac:dyDescent="0.25">
+    <row r="6" spans="3:13" x14ac:dyDescent="0.25">
       <c r="C6" s="2">
         <v>913.46</v>
       </c>
@@ -652,6 +684,496 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0027F471-9B04-4A6B-B21C-CFABD149F1B5}">
+  <dimension ref="A1:P11"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="11" max="11" width="27.28515625" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="17" customWidth="1"/>
+    <col min="13" max="13" width="17.28515625" customWidth="1"/>
+    <col min="16" max="16" width="11.85546875" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="K1" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="L1" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="M1" s="1" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="2" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A2" s="4">
+        <v>21</v>
+      </c>
+      <c r="B2" s="4">
+        <v>1167.1300000000001</v>
+      </c>
+      <c r="C2" s="4">
+        <v>1167.05</v>
+      </c>
+      <c r="D2" s="5">
+        <f>AVERAGE(B2:C2)</f>
+        <v>1167.0900000000001</v>
+      </c>
+      <c r="E2" s="4">
+        <v>1167.0899999999999</v>
+      </c>
+      <c r="F2" s="4">
+        <v>393.87</v>
+      </c>
+      <c r="G2" s="4">
+        <v>393.35</v>
+      </c>
+      <c r="H2" s="5">
+        <f>AVERAGE(F2:G2)</f>
+        <v>393.61</v>
+      </c>
+      <c r="I2" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="J2" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="K2" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="L2" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="M2" s="4">
+        <v>6.53</v>
+      </c>
+      <c r="P2" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="3" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A3" s="4">
+        <v>21</v>
+      </c>
+      <c r="B3" s="4">
+        <v>1171.6099999999999</v>
+      </c>
+      <c r="C3" s="4">
+        <v>1171.8800000000001</v>
+      </c>
+      <c r="D3" s="5">
+        <f t="shared" ref="D3:D11" si="0">AVERAGE(B3:C3)</f>
+        <v>1171.7449999999999</v>
+      </c>
+      <c r="E3" s="4">
+        <v>1171.75</v>
+      </c>
+      <c r="F3" s="4">
+        <v>397.57</v>
+      </c>
+      <c r="G3" s="4">
+        <v>402.71</v>
+      </c>
+      <c r="H3" s="5">
+        <f t="shared" ref="H3:H11" si="1">AVERAGE(F3:G3)</f>
+        <v>400.14</v>
+      </c>
+      <c r="I3" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="J3" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="K3" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="L3" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="M3" s="4">
+        <v>6.96</v>
+      </c>
+    </row>
+    <row r="4" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A4" s="4">
+        <v>21</v>
+      </c>
+      <c r="B4" s="4">
+        <v>1177.93</v>
+      </c>
+      <c r="C4" s="4">
+        <v>1178.3699999999999</v>
+      </c>
+      <c r="D4" s="5">
+        <f t="shared" si="0"/>
+        <v>1178.1500000000001</v>
+      </c>
+      <c r="E4" s="4">
+        <v>1178.1500000000001</v>
+      </c>
+      <c r="F4" s="4">
+        <v>404.09</v>
+      </c>
+      <c r="G4" s="4">
+        <v>403.96</v>
+      </c>
+      <c r="H4" s="5">
+        <f t="shared" si="1"/>
+        <v>404.02499999999998</v>
+      </c>
+      <c r="I4" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="J4" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="K4" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="L4" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="M4" s="4">
+        <v>6.61</v>
+      </c>
+    </row>
+    <row r="5" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A5" s="4">
+        <v>21</v>
+      </c>
+      <c r="B5" s="4">
+        <v>1181.04</v>
+      </c>
+      <c r="C5" s="4">
+        <v>1180.69</v>
+      </c>
+      <c r="D5" s="5">
+        <f t="shared" si="0"/>
+        <v>1180.865</v>
+      </c>
+      <c r="E5" s="4">
+        <v>1180.8699999999999</v>
+      </c>
+      <c r="F5" s="4">
+        <v>405.26</v>
+      </c>
+      <c r="G5" s="4">
+        <v>404.67</v>
+      </c>
+      <c r="H5" s="5">
+        <f t="shared" si="1"/>
+        <v>404.96500000000003</v>
+      </c>
+      <c r="I5" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="J5" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="K5" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="L5" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="M5" s="4">
+        <v>6.49</v>
+      </c>
+    </row>
+    <row r="6" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A6" s="4">
+        <v>21</v>
+      </c>
+      <c r="B6" s="4">
+        <v>1177.67</v>
+      </c>
+      <c r="C6" s="4">
+        <v>1177.26</v>
+      </c>
+      <c r="D6" s="5">
+        <f t="shared" si="0"/>
+        <v>1177.4650000000001</v>
+      </c>
+      <c r="E6" s="4">
+        <v>1177.47</v>
+      </c>
+      <c r="F6" s="4">
+        <v>403.69</v>
+      </c>
+      <c r="G6" s="4">
+        <v>404.48</v>
+      </c>
+      <c r="H6" s="5">
+        <f t="shared" si="1"/>
+        <v>404.08500000000004</v>
+      </c>
+      <c r="I6" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="J6" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="K6" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="L6" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="M6" s="4">
+        <v>6.45</v>
+      </c>
+    </row>
+    <row r="7" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A7" s="4">
+        <v>-35</v>
+      </c>
+      <c r="B7" s="4">
+        <v>1131.94</v>
+      </c>
+      <c r="C7" s="4">
+        <v>1131.53</v>
+      </c>
+      <c r="D7" s="5">
+        <f t="shared" si="0"/>
+        <v>1131.7350000000001</v>
+      </c>
+      <c r="E7" s="4">
+        <v>1131.74</v>
+      </c>
+      <c r="F7" s="5">
+        <v>380.64789999999999</v>
+      </c>
+      <c r="G7" s="5">
+        <v>379.59679999999997</v>
+      </c>
+      <c r="H7" s="5">
+        <f t="shared" si="1"/>
+        <v>380.12234999999998</v>
+      </c>
+      <c r="I7" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="J7" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="K7" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="L7" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="M7" s="4">
+        <v>6.59</v>
+      </c>
+    </row>
+    <row r="8" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A8" s="4">
+        <v>-35</v>
+      </c>
+      <c r="B8" s="4">
+        <v>1131.19</v>
+      </c>
+      <c r="C8" s="4">
+        <v>1130.3599999999999</v>
+      </c>
+      <c r="D8" s="5">
+        <f t="shared" si="0"/>
+        <v>1130.7750000000001</v>
+      </c>
+      <c r="E8" s="4">
+        <v>1130.78</v>
+      </c>
+      <c r="F8" s="5">
+        <v>376.2278</v>
+      </c>
+      <c r="G8" s="5">
+        <v>377.19959999999998</v>
+      </c>
+      <c r="H8" s="5">
+        <f t="shared" si="1"/>
+        <v>376.71370000000002</v>
+      </c>
+      <c r="I8" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="J8" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="K8" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="L8" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="M8" s="4">
+        <v>6.96</v>
+      </c>
+    </row>
+    <row r="9" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A9" s="4">
+        <v>-35</v>
+      </c>
+      <c r="B9" s="4">
+        <v>1129.55</v>
+      </c>
+      <c r="C9" s="4">
+        <v>1129.1500000000001</v>
+      </c>
+      <c r="D9" s="5">
+        <f t="shared" si="0"/>
+        <v>1129.3499999999999</v>
+      </c>
+      <c r="E9" s="4">
+        <v>1129.3499999999999</v>
+      </c>
+      <c r="F9" s="5">
+        <v>373.8408</v>
+      </c>
+      <c r="G9" s="5">
+        <v>383.2063</v>
+      </c>
+      <c r="H9" s="5">
+        <f t="shared" si="1"/>
+        <v>378.52355</v>
+      </c>
+      <c r="I9" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="J9" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="K9" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="L9" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="M9" s="4">
+        <v>7.19</v>
+      </c>
+    </row>
+    <row r="10" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A10" s="4">
+        <v>-35</v>
+      </c>
+      <c r="B10" s="4">
+        <v>1136.04</v>
+      </c>
+      <c r="C10" s="4">
+        <v>1135.4100000000001</v>
+      </c>
+      <c r="D10" s="5">
+        <f t="shared" si="0"/>
+        <v>1135.7249999999999</v>
+      </c>
+      <c r="E10" s="4">
+        <v>1135.73</v>
+      </c>
+      <c r="F10" s="5">
+        <v>383.2817</v>
+      </c>
+      <c r="G10" s="5">
+        <v>387.1352</v>
+      </c>
+      <c r="H10" s="5">
+        <f t="shared" si="1"/>
+        <v>385.20844999999997</v>
+      </c>
+      <c r="I10" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="J10" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="K10" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="L10" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="M10" s="4">
+        <v>7.13</v>
+      </c>
+    </row>
+    <row r="11" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A11" s="4">
+        <v>-35</v>
+      </c>
+      <c r="B11" s="4">
+        <v>1126.02</v>
+      </c>
+      <c r="C11" s="4">
+        <v>1125.3599999999999</v>
+      </c>
+      <c r="D11" s="5">
+        <f t="shared" si="0"/>
+        <v>1125.69</v>
+      </c>
+      <c r="E11" s="4">
+        <v>1125.69</v>
+      </c>
+      <c r="F11" s="5">
+        <v>372.94760000000002</v>
+      </c>
+      <c r="G11" s="5">
+        <v>374.0643</v>
+      </c>
+      <c r="H11" s="5">
+        <f t="shared" si="1"/>
+        <v>373.50594999999998</v>
+      </c>
+      <c r="I11" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="J11" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="K11" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="L11" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="M11" s="4">
+        <v>6.44</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{298C37D3-CA03-4C85-9F91-82C86E07EA81}">
   <dimension ref="A1:Z1"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -665,28 +1187,28 @@
   <sheetData>
     <row r="1" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C1" t="s">
+        <v>13</v>
+      </c>
+      <c r="D1" t="s">
+        <v>14</v>
+      </c>
+      <c r="E1" t="s">
+        <v>12</v>
+      </c>
+      <c r="V1" t="s">
         <v>11</v>
       </c>
-      <c r="C1" t="s">
-        <v>14</v>
-      </c>
-      <c r="D1" t="s">
+      <c r="X1" t="s">
         <v>15</v>
       </c>
-      <c r="E1" t="s">
-        <v>13</v>
-      </c>
-      <c r="V1" t="s">
-        <v>12</v>
-      </c>
-      <c r="X1" t="s">
+      <c r="Y1" t="s">
         <v>16</v>
       </c>
-      <c r="Y1" t="s">
+      <c r="Z1" t="s">
         <v>17</v>
-      </c>
-      <c r="Z1" t="s">
-        <v>18</v>
       </c>
     </row>
   </sheetData>

</xml_diff>